<commit_message>
Add vga_lcd scaled cases to progression workbook
</commit_message>
<xml_diff>
--- a/doc/presentation-data/descriptor_progression_cumulative_rtx5090_k1m.xlsx
+++ b/doc/presentation-data/descriptor_progression_cumulative_rtx5090_k1m.xlsx
@@ -319,7 +319,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -489,8 +489,52 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>vga_lcd x8</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>14.528 ms</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>13.170 ms (1.103×)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>10.205 ms (1.424×)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>vga_lcd x16</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>14.861 ms</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>12.434 ms (1.195×)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>10.389 ms (1.430×)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Speedups below 1× indicate a slowdown.</t>
         </is>

</xml_diff>

<commit_message>
Add des_perf and vga_lcd original cases to workbook
</commit_message>
<xml_diff>
--- a/doc/presentation-data/descriptor_progression_cumulative_rtx5090_k1m.xlsx
+++ b/doc/presentation-data/descriptor_progression_cumulative_rtx5090_k1m.xlsx
@@ -11,7 +11,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -115,8 +115,52 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>des_perf</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>26.745 ms</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>27.503 ms (0.972×)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>29.022 ms (0.922×)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>vga_lcd</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>7.994 ms</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>8.395 ms (0.952×)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>9.360 ms (0.854×)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Speedups below 1× indicate a slowdown.</t>
         </is>

</xml_diff>